<commit_message>
Updated BBP Sel IDE test cases to update the Cardit Card Expiration Year
</commit_message>
<xml_diff>
--- a/KatalonData/IWPBootstrapData/VRelayPaymentsCC_27.xlsx
+++ b/KatalonData/IWPBootstrapData/VRelayPaymentsCC_27.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="83">
   <si>
     <t>Result</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t>Tue Nov 18 21:54:40 IST 2025</t>
+  </si>
+  <si>
+    <t>Thu Jan 29 14:40:52 EST 2026</t>
   </si>
 </sst>
 </file>
@@ -664,7 +667,7 @@
         <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">

</xml_diff>

<commit_message>
Added Test Cases in IWP 2.7 Bootstrap
</commit_message>
<xml_diff>
--- a/KatalonData/IWPBootstrapData/VRelayPaymentsCC_27.xlsx
+++ b/KatalonData/IWPBootstrapData/VRelayPaymentsCC_27.xlsx
@@ -1,23 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T476640\Documents\VPS_Katalon\VPS-Katalon\KatalonData\IWPBootstrapData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\IWPBootstrapData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{A3A8FEEC-D608-4C6D-8837-2216312FCFDC}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr documentId="13_ncr:1_{3D90974E-318F-4435-8142-EECE88F4B131}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView activeTab="4" windowHeight="10420" windowWidth="19420" xWindow="-110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-110"/>
+    <workbookView activeTab="2" windowHeight="12456" windowWidth="23256" xWindow="-108" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-108"/>
   </bookViews>
   <sheets>
-    <sheet name="PayNowCC_27" r:id="rId1" sheetId="1"/>
-    <sheet name="PayNowSCFCC_27" r:id="rId2" sheetId="2"/>
-    <sheet name="PayNowDCFCC_27" r:id="rId3" sheetId="3"/>
-    <sheet name="CCDeferredCC_27" r:id="rId4" sheetId="4"/>
-    <sheet name="CMCAutopayCC_27" r:id="rId5" sheetId="5"/>
+    <sheet name="PayNowCCNoCF" r:id="rId1" sheetId="6"/>
+    <sheet name="PayNowCC_27" r:id="rId2" sheetId="1"/>
+    <sheet name="VerifyPaymentConfPayNowCC" r:id="rId3" sheetId="21"/>
+    <sheet name="ModifyPaymentsCC1" r:id="rId4" sheetId="15"/>
+    <sheet name="ModifyPaymentsCC2" r:id="rId5" sheetId="16"/>
+    <sheet name="NoModifyAmountCC" r:id="rId6" sheetId="17"/>
+    <sheet name="NoModifyBillingAddressCC" r:id="rId7" sheetId="18"/>
+    <sheet name="PayNowSCFCC_27" r:id="rId8" sheetId="2"/>
+    <sheet name="SCFCCVerbiage" r:id="rId9" sheetId="20"/>
+    <sheet name="PayNowDCFCC_27" r:id="rId10" sheetId="3"/>
+    <sheet name="DCFCCVerbiage" r:id="rId11" sheetId="19"/>
+    <sheet name="CCDeferredCC_27" r:id="rId12" sheetId="4"/>
+    <sheet name="CMCAutopayCC_27" r:id="rId13" sheetId="5"/>
+    <sheet name="CancelStaticTextAutopayCC" r:id="rId14" sheetId="7"/>
+    <sheet name="CancelSuccessAutopayCC" r:id="rId15" sheetId="8"/>
+    <sheet name="CancelStaticTextDeferredCC" r:id="rId16" sheetId="9"/>
+    <sheet name="CancelSuccessDeferredCC" r:id="rId17" sheetId="10"/>
+    <sheet name="ModifyStaticTextAutopayCC" r:id="rId18" sheetId="11"/>
+    <sheet name="ModifySuccessAutopayCC" r:id="rId19" sheetId="12"/>
+    <sheet name="ModifyStaticTextDeferredCC" r:id="rId20" sheetId="13"/>
+    <sheet name="ModifySuccessDeferredCC" r:id="rId21" sheetId="14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="54">
   <si>
     <t>Result</t>
   </si>
@@ -106,325 +122,91 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Sat Jan 18 00:17:42 IST 2025</t>
-  </si>
-  <si>
     <t>832</t>
   </si>
   <si>
     <t>888</t>
   </si>
   <si>
-    <t>Thu Jan 23 14:53:56 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jan 23 15:01:50 IST 2025</t>
-  </si>
-  <si>
     <t>29/08/2029</t>
   </si>
   <si>
-    <t>Thu Jan 23 17:27:15 IST 2025</t>
-  </si>
-  <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>Tue Dec 17 17:02:38 IST 2024</t>
-  </si>
-  <si>
     <t>19</t>
   </si>
   <si>
+    <t>Sat Feb 28 14:42:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Feb 28 14:46:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 03 20:47:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Mar 04 00:22:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Mar 04 18:13:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Mar 26 21:06:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 27 18:47:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 27 19:38:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 27 20:13:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 27 20:55:43 IST 2026</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>979</t>
+  </si>
+  <si>
+    <t>Wed Apr 01 22:18:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Apr 02 20:53:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Apr 03 19:30:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Apr 03 19:33:21 IST 2026</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Wed Jan 29 17:30:11 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Feb 26 16:00:10 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Feb 26 16:07:25 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Feb 26 16:17:17 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Feb 26 16:25:18 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Feb 26 16:29:57 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Feb 27 20:29:37 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Feb 27 20:35:43 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Feb 28 13:16:18 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Feb 28 13:27:07 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Feb 28 13:37:30 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 05 14:32:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 05 14:33:23 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 05 14:36:58 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 05 18:10:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 26 14:53:19 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 26 15:03:13 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 26 15:08:57 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Mar 26 15:13:28 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Apr 07 21:05:15 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Apr 07 21:15:14 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Apr 07 21:21:04 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Apr 07 21:25:37 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Jun 02 21:35:38 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Jun 02 21:43:01 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Jun 02 21:46:44 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Jun 02 21:49:42 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Jun 04 12:30:51 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Jun 04 12:55:00 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Jun 04 12:56:04 IST 2025</t>
-  </si>
-  <si>
-    <t>Wed Jun 04 13:29:59 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jun 05 11:45:24 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jun 05 11:53:15 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jun 05 11:57:14 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jun 05 12:00:19 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Aug 29 23:59:23 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Aug 30 00:08:24 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Aug 30 00:12:10 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Aug 30 00:15:44 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Aug 30 00:18:21 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 08 13:43:08 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 08 13:49:13 IST 2025</t>
-  </si>
-  <si>
-    <t>Sat Nov 08 13:53:29 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 13 21:27:27 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Nov 13 21:44:26 IST 2025</t>
-  </si>
-  <si>
-    <t>Tue Nov 18 21:54:40 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Jan 29 14:40:52 EST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 03 21:23:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Feb 04 20:05:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 22:31:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 22:55:53 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 23:03:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 23:07:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 23:11:13 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 23:47:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Feb 05 23:55:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 06 00:03:00 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 06 00:07:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 06 00:11:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 06 18:41:43 IST 2026</t>
-  </si>
-  <si>
-    <t>Mon Feb 09 22:00:59 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 01:03:08 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 01:12:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 01:22:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 01:28:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 01:32:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Feb 10 19:39:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 02:18:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 02:28:28 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 02:37:41 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 02:46:40 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 02:54:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 06:42:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 06:50:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 06:54:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 06:58:15 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 19:00:55 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 20:52:03 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 20:57:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:02:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:08:12 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Feb 20 21:25:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 21 08:00:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 21 08:08:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 21 08:15:38 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 21 08:20:03 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 21 08:23:45 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 28 14:15:36 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 28 14:25:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 28 14:35:14 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 28 14:42:25 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Feb 28 14:46:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 03 20:37:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 03 20:47:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 00:22:15 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Mar 04 18:13:47 IST 2026</t>
+    <t>Mon Apr 06 21:55:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 06 21:57:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 06 22:11:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Apr 06 22:14:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 08 19:00:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 08 19:04:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Apr 08 19:09:28 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -761,11 +543,1050 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F7A018-07CA-4DE2-85D2-C45310919A6D}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F14611B2-272D-4F6C-A3A3-34625CF21E5C}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFF4BB81-CC08-4091-9D95-3A4A11E173EE}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924AD824-C93A-4DEC-A40B-651CCF250E75}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.77734375" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row ht="28.8" r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26DA0F3-1CAA-4554-B84A-57402F442697}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6859EFA-971B-46EF-9F88-19ADA00CDDC2}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4B4F343-DA62-4980-9834-419A05CC33C3}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E8C958B-BC9A-44BC-84D9-4487E068BDBA}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.77734375" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row ht="28.8" r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD46E377-6BD6-4BA8-BB7B-7095CAEE12C3}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.77734375" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row ht="28.8" r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{502AF05A-5E83-4891-B6D4-3A99DCDD7B93}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D64F9E7-8E19-4FF9-858F-B27AAD9E9DD1}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row ht="29" r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -809,12 +1630,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -857,12 +1678,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A599422F-DB1C-494D-AC7A-FABC7A55F2B3}">
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FF5417-5A97-4FF0-B4A6-4CB3ACCC5E12}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.77734375" collapsed="true"/>
+  </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -906,12 +1730,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>127</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -921,7 +1745,7 @@
         <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>16</v>
@@ -938,7 +1762,108 @@
       <c r="K2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="1"/>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4A1512-11EF-4F9D-8705-BB77A40DA376}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.77734375" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row ht="28.8" r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="M2" s="1" t="s">
         <v>21</v>
       </c>
@@ -952,11 +1877,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F14611B2-272D-4F6C-A3A3-34625CF21E5C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F387F6-118B-48DC-9C79-B9D10422FE4D}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row ht="29" r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1000,12 +1925,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -1015,7 +1940,7 @@
         <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>16</v>
@@ -1046,14 +1971,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924AD824-C93A-4DEC-A40B-651CCF250E75}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{122661BC-EB0E-415D-9F4C-17C6AACD5339}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="24.81640625" collapsed="true"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row ht="29" r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1097,13 +2019,7 @@
         <v>13</v>
       </c>
     </row>
-    <row ht="29" r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>131</v>
-      </c>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
         <v>14</v>
@@ -1127,11 +2043,9 @@
         <v>19</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>30</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="L2" s="1"/>
       <c r="M2" s="1" t="s">
         <v>21</v>
       </c>
@@ -1145,11 +2059,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26DA0F3-1CAA-4554-B84A-57402F442697}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00532F1A-916F-4150-88F2-B68490CEFE46}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row ht="29" r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1193,19 +2107,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>129</v>
-      </c>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>23</v>
@@ -1213,7 +2121,381 @@
       <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01D345C4-0731-4594-B067-756A7E19A715}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BA9A57-C3C6-46D0-A1CE-2333157B7279}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A599422F-DB1C-494D-AC7A-FABC7A55F2B3}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C8C373-558A-4744-952F-549562AC4B84}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row ht="28.8" r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="I2" s="1" t="s">
         <v>18</v>
       </c>

</xml_diff>